<commit_message>
Revised cover reading guide etc.
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Retail_Peer_Benchmarking.xlsx
+++ b/output/Retail_Peer_Benchmarking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude_Projects\retail-peer-benchmarking\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D723968E-169C-4CC6-90A0-42D6D11B2036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762D09B9-158D-4D8B-803A-F0A58008AD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="948" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -269,7 +269,7 @@
     <t>Start here</t>
   </si>
   <si>
-    <t>Executive Summary – the three questions, each answered in one bold line, followed by the evidence. Five minutes.</t>
+    <t>Executive Summary – the three questions, each answered in one bold line, followed by the evidence.</t>
   </si>
   <si>
     <t>Then</t>
@@ -2667,7 +2667,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7887-4E4E-9E06-D69A0794FE8C}"/>
+              <c16:uniqueId val="{00000000-4DE3-44C6-A156-14BBE990BBDC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2680,8 +2680,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1442829296"/>
-        <c:axId val="1377578992"/>
+        <c:axId val="1379402736"/>
+        <c:axId val="792016016"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2803,7 +2803,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7887-4E4E-9E06-D69A0794FE8C}"/>
+              <c16:uniqueId val="{00000001-4DE3-44C6-A156-14BBE990BBDC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2924,7 +2924,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-7887-4E4E-9E06-D69A0794FE8C}"/>
+              <c16:uniqueId val="{00000002-4DE3-44C6-A156-14BBE990BBDC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3045,7 +3045,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-7887-4E4E-9E06-D69A0794FE8C}"/>
+              <c16:uniqueId val="{00000003-4DE3-44C6-A156-14BBE990BBDC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3166,7 +3166,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-7887-4E4E-9E06-D69A0794FE8C}"/>
+              <c16:uniqueId val="{00000004-4DE3-44C6-A156-14BBE990BBDC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3287,7 +3287,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-7887-4E4E-9E06-D69A0794FE8C}"/>
+              <c16:uniqueId val="{00000005-4DE3-44C6-A156-14BBE990BBDC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3364,7 +3364,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1377578992"/>
+        <c:axId val="792016016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3399,12 +3399,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1442829296"/>
+        <c:crossAx val="1379402736"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1442829296"/>
+        <c:axId val="1379402736"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3414,7 +3414,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1377578992"/>
+        <c:crossAx val="792016016"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3584,7 +3584,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EBBA-4106-BDFD-553F7ABB8764}"/>
+              <c16:uniqueId val="{00000000-1E8E-4095-837F-95A448011140}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3597,8 +3597,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1442831616"/>
-        <c:axId val="1377575152"/>
+        <c:axId val="1379405984"/>
+        <c:axId val="792036176"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -3720,7 +3720,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-EBBA-4106-BDFD-553F7ABB8764}"/>
+              <c16:uniqueId val="{00000001-1E8E-4095-837F-95A448011140}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3841,7 +3841,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-EBBA-4106-BDFD-553F7ABB8764}"/>
+              <c16:uniqueId val="{00000002-1E8E-4095-837F-95A448011140}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3962,7 +3962,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-EBBA-4106-BDFD-553F7ABB8764}"/>
+              <c16:uniqueId val="{00000003-1E8E-4095-837F-95A448011140}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4083,7 +4083,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-EBBA-4106-BDFD-553F7ABB8764}"/>
+              <c16:uniqueId val="{00000004-1E8E-4095-837F-95A448011140}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4160,7 +4160,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1377575152"/>
+        <c:axId val="792036176"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4195,12 +4195,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1442831616"/>
+        <c:crossAx val="1379405984"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1442831616"/>
+        <c:axId val="1379405984"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4210,7 +4210,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1377575152"/>
+        <c:crossAx val="792036176"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -4380,7 +4380,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-50A7-4FCB-AAE4-155A87FFBD81}"/>
+              <c16:uniqueId val="{00000000-19AE-4859-B537-9CB63D8246F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4393,8 +4393,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1442833472"/>
-        <c:axId val="1377569392"/>
+        <c:axId val="1376477344"/>
+        <c:axId val="792053936"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4516,7 +4516,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-50A7-4FCB-AAE4-155A87FFBD81}"/>
+              <c16:uniqueId val="{00000001-19AE-4859-B537-9CB63D8246F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4637,7 +4637,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-50A7-4FCB-AAE4-155A87FFBD81}"/>
+              <c16:uniqueId val="{00000002-19AE-4859-B537-9CB63D8246F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4758,7 +4758,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-50A7-4FCB-AAE4-155A87FFBD81}"/>
+              <c16:uniqueId val="{00000003-19AE-4859-B537-9CB63D8246F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4879,7 +4879,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-50A7-4FCB-AAE4-155A87FFBD81}"/>
+              <c16:uniqueId val="{00000004-19AE-4859-B537-9CB63D8246F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5000,7 +5000,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-50A7-4FCB-AAE4-155A87FFBD81}"/>
+              <c16:uniqueId val="{00000005-19AE-4859-B537-9CB63D8246F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5077,7 +5077,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1377569392"/>
+        <c:axId val="792053936"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5112,12 +5112,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1442833472"/>
+        <c:crossAx val="1376477344"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1442833472"/>
+        <c:axId val="1376477344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5127,7 +5127,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1377569392"/>
+        <c:crossAx val="792053936"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -5297,7 +5297,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A0DC-4685-9046-397B8D0D78E3}"/>
+              <c16:uniqueId val="{00000000-43EF-44D9-B843-4D43C1342D8F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5310,8 +5310,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1436528352"/>
-        <c:axId val="1377571312"/>
+        <c:axId val="1379403664"/>
+        <c:axId val="792046736"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -5433,7 +5433,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A0DC-4685-9046-397B8D0D78E3}"/>
+              <c16:uniqueId val="{00000001-43EF-44D9-B843-4D43C1342D8F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5554,7 +5554,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-A0DC-4685-9046-397B8D0D78E3}"/>
+              <c16:uniqueId val="{00000002-43EF-44D9-B843-4D43C1342D8F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5675,7 +5675,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-A0DC-4685-9046-397B8D0D78E3}"/>
+              <c16:uniqueId val="{00000003-43EF-44D9-B843-4D43C1342D8F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5796,7 +5796,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-A0DC-4685-9046-397B8D0D78E3}"/>
+              <c16:uniqueId val="{00000004-43EF-44D9-B843-4D43C1342D8F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5873,7 +5873,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1377571312"/>
+        <c:axId val="792046736"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -5908,12 +5908,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1436528352"/>
+        <c:crossAx val="1379403664"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1436528352"/>
+        <c:axId val="1379403664"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5923,7 +5923,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1377571312"/>
+        <c:crossAx val="792046736"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6093,7 +6093,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D284-4468-B2E2-B604EE5BDBDB}"/>
+              <c16:uniqueId val="{00000000-A446-491F-A251-4E870EE46D35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6106,8 +6106,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1442830688"/>
-        <c:axId val="1377587632"/>
+        <c:axId val="1379408768"/>
+        <c:axId val="792076976"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6229,7 +6229,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D284-4468-B2E2-B604EE5BDBDB}"/>
+              <c16:uniqueId val="{00000001-A446-491F-A251-4E870EE46D35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6350,7 +6350,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-D284-4468-B2E2-B604EE5BDBDB}"/>
+              <c16:uniqueId val="{00000002-A446-491F-A251-4E870EE46D35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6471,7 +6471,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-D284-4468-B2E2-B604EE5BDBDB}"/>
+              <c16:uniqueId val="{00000003-A446-491F-A251-4E870EE46D35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6592,7 +6592,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-D284-4468-B2E2-B604EE5BDBDB}"/>
+              <c16:uniqueId val="{00000004-A446-491F-A251-4E870EE46D35}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6669,7 +6669,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1377587632"/>
+        <c:axId val="792076976"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -6704,12 +6704,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1442830688"/>
+        <c:crossAx val="1379408768"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1442830688"/>
+        <c:axId val="1379408768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6719,7 +6719,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1377587632"/>
+        <c:crossAx val="792076976"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -6889,7 +6889,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B141-4CB8-8252-704D0B7B2D52}"/>
+              <c16:uniqueId val="{00000000-3FD4-4619-BF2B-B9938DAB6414}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6902,8 +6902,8 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="0"/>
-        <c:axId val="1925784176"/>
-        <c:axId val="1377486832"/>
+        <c:axId val="1379406448"/>
+        <c:axId val="791971856"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -7025,7 +7025,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B141-4CB8-8252-704D0B7B2D52}"/>
+              <c16:uniqueId val="{00000001-3FD4-4619-BF2B-B9938DAB6414}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7146,7 +7146,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-B141-4CB8-8252-704D0B7B2D52}"/>
+              <c16:uniqueId val="{00000002-3FD4-4619-BF2B-B9938DAB6414}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7267,7 +7267,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-B141-4CB8-8252-704D0B7B2D52}"/>
+              <c16:uniqueId val="{00000003-3FD4-4619-BF2B-B9938DAB6414}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7388,7 +7388,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-B141-4CB8-8252-704D0B7B2D52}"/>
+              <c16:uniqueId val="{00000004-3FD4-4619-BF2B-B9938DAB6414}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7509,7 +7509,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-B141-4CB8-8252-704D0B7B2D52}"/>
+              <c16:uniqueId val="{00000005-3FD4-4619-BF2B-B9938DAB6414}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7586,7 +7586,7 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1377486832"/>
+        <c:axId val="791971856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -7621,12 +7621,12 @@
             </a:ext>
           </a:extLst>
         </c:spPr>
-        <c:crossAx val="1925784176"/>
+        <c:crossAx val="1379406448"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="1925784176"/>
+        <c:axId val="1379406448"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7636,7 +7636,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1377486832"/>
+        <c:crossAx val="791971856"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>

</xml_diff>